<commit_message>
App: nút ⓘ giới thiệu chung ở trang menu Sản xuất, Khai báo, Báo cáo; thêm ⓘ vào thanh chức năng của Khai báo (D123)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Agricovi_Mo_hinh_doanh_thu_v2.xlsx
+++ b/docs/Agricovi_Mo_hinh_doanh_thu_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AgriCo\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C6FAAF0-4AF2-447A-BDB5-1F1BB6FB891A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA0A9FB-9F9C-43A0-876B-90DAD7C4E872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hướng dẫn" sheetId="1" r:id="rId1"/>
@@ -994,7 +994,7 @@
         <v>600</v>
       </c>
       <c r="D16" s="8">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="E16" t="s">
         <v>30</v>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="D6" s="12">
         <f>'Giả định'!D16*D4</f>
-        <v>9000000000</v>
+        <v>7200000000</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="D8" s="14">
         <f>D6+D7</f>
-        <v>13140000000</v>
+        <v>11340000000</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="D15" s="14">
         <f>D8+D14</f>
-        <v>13140000000</v>
+        <v>11340000000</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="D21" s="12">
         <f>'Giả định'!D44+'Giả định'!D16*'Giả định'!D45+'Giả định'!D17*'Giả định'!D46</f>
-        <v>610000000</v>
+        <v>586000000</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="D22" s="12">
         <f>D8*'Giả định'!D47</f>
-        <v>197100000</v>
+        <v>170100000</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="D25" s="12">
         <f>SUM(D18:D24)*'Giả định'!D50</f>
-        <v>785510000</v>
+        <v>780410000</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="D26" s="14">
         <f>SUM(D18:D25)</f>
-        <v>8640610000</v>
+        <v>8584510000</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D27" s="14">
         <f>D15-D26</f>
-        <v>4499390000</v>
+        <v>2755490000</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="D28" s="12">
         <f>C28+D27</f>
-        <v>6245315000</v>
+        <v>4501415000</v>
       </c>
     </row>
     <row r="29" spans="1:4">

</xml_diff>